<commit_message>
#26 D6 and C13 update in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client-BOM-Solenoid-Switching-Board-v1.0.xlsx
+++ b/Design Files/Solenoid-Switching-Board-v1.0/BOM/Client-BOM-Solenoid-Switching-Board-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="97">
   <si>
     <t>#</t>
   </si>
@@ -117,9 +117,6 @@
     <t>CAP CER 0.1UF 50V X5R 0603</t>
   </si>
   <si>
-    <t>CAP ALUM 220UF 20% 50V SMD</t>
-  </si>
-  <si>
     <t>SMC(DO-214AB) Diodes - Fast Recovery Rectifiers ROHS</t>
   </si>
   <si>
@@ -168,9 +165,6 @@
     <t>Cap-0603</t>
   </si>
   <si>
-    <t>UCD-220uF-10mmDia</t>
-  </si>
-  <si>
     <t>SMC</t>
   </si>
   <si>
@@ -198,9 +192,6 @@
     <t>CC0603KRX5R9BB104</t>
   </si>
   <si>
-    <t>UCD1H221MNL1GS</t>
-  </si>
-  <si>
     <t>MURS360T3G</t>
   </si>
   <si>
@@ -240,9 +231,6 @@
     <t>Yageo</t>
   </si>
   <si>
-    <t>Nichicon</t>
-  </si>
-  <si>
     <t>FUXINSEMI</t>
   </si>
   <si>
@@ -270,9 +258,6 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>220uF</t>
-  </si>
-  <si>
     <t>2.2K</t>
   </si>
   <si>
@@ -298,6 +283,33 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 60V 5A SMA</t>
+  </si>
+  <si>
+    <t>SMA</t>
+  </si>
+  <si>
+    <t>SS56</t>
+  </si>
+  <si>
+    <t>MDD</t>
+  </si>
+  <si>
+    <t>100uF 50V ±20% SMD,D6.3xL7.7mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
+  </si>
+  <si>
+    <t>RVT1H101M0607</t>
+  </si>
+  <si>
+    <t>ROQANG</t>
+  </si>
+  <si>
+    <t>100uF</t>
   </si>
 </sst>
 </file>
@@ -790,7 +802,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -803,6 +815,7 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -833,22 +846,22 @@
         <v>29</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -867,16 +880,16 @@
         <v>30</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="J3" s="7">
         <v>4</v>
@@ -886,7 +899,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B18" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B19" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -899,23 +912,23 @@
         <v>31</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="J4" s="9">
         <v>9</v>
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
@@ -928,19 +941,19 @@
         <v>15</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>32</v>
+        <v>93</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>73</v>
+        <v>95</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
@@ -960,19 +973,19 @@
         <v>16</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
@@ -992,376 +1005,405 @@
         <v>17</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
       </c>
       <c r="K7" s="7"/>
     </row>
-    <row r="8" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="11">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>5</v>
+      <c r="B8" s="11"/>
+      <c r="C8" s="12" t="s">
+        <v>4</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>52</v>
-      </c>
       <c r="H8" s="9" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="J8" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
-        <f>ROW(B9) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>36</v>
+      <c r="C9" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>76</v>
+        <v>86</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>71</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J9" s="7">
-        <v>1</v>
-      </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="J9" s="9">
+        <v>4</v>
+      </c>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B10) - ROW($B$2)</f>
         <v>8</v>
       </c>
-      <c r="C10" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>37</v>
+      <c r="C10" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>35</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>77</v>
+        <v>86</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J10" s="9">
+        <v>87</v>
+      </c>
+      <c r="J10" s="7">
         <v>1</v>
       </c>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
-        <f>ROW(B11) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>38</v>
+      <c r="C11" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="G11" s="8">
-        <v>1715721</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>78</v>
+        <v>86</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J11" s="7">
+        <v>87</v>
+      </c>
+      <c r="J11" s="9">
         <v>1</v>
       </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B12) - ROW($B$2)</f>
         <v>10</v>
       </c>
-      <c r="C12" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>79</v>
+      <c r="C12" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G12" s="8">
+        <v>1715721</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" s="9">
-        <v>4</v>
-      </c>
-      <c r="K12" s="9"/>
+        <v>87</v>
+      </c>
+      <c r="J12" s="7">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7"/>
     </row>
     <row r="13" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
-        <f>ROW(B13) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>79</v>
+      <c r="D13" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>75</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J13" s="7">
-        <v>5</v>
-      </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>87</v>
+      </c>
+      <c r="J13" s="9">
+        <v>4</v>
+      </c>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B14) - ROW($B$2)</f>
         <v>12</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>72</v>
+        <v>9</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>75</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="J14" s="9">
-        <v>4</v>
-      </c>
-      <c r="K14" s="9"/>
+        <v>87</v>
+      </c>
+      <c r="J14" s="7">
+        <v>5</v>
+      </c>
+      <c r="K14" s="7"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
-        <f>ROW(B15) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="J15" s="7">
+      <c r="D15" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="J15" s="9">
         <v>4</v>
       </c>
-      <c r="K15" s="7"/>
+      <c r="K15" s="9"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B16) - ROW($B$2)</f>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="J16" s="9">
-        <v>8</v>
-      </c>
-      <c r="K16" s="9"/>
+      <c r="D16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="J16" s="7">
+        <v>4</v>
+      </c>
+      <c r="K16" s="7"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
-        <f>ROW(B17) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="J17" s="7">
-        <v>5</v>
-      </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="J17" s="9">
+        <v>8</v>
+      </c>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
+        <f>ROW(B18) - ROW($B$2)</f>
+        <v>16</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="J18" s="7">
+        <v>5</v>
+      </c>
+      <c r="K18" s="7"/>
+    </row>
+    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="11">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C18" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D19" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="J18" s="9">
+      <c r="E19" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="J19" s="9">
         <v>4</v>
       </c>
-      <c r="K18" s="9"/>
+      <c r="K19" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>